<commit_message>
feat: add pipeline's results
</commit_message>
<xml_diff>
--- a/data/final/tables/bootstrap_summary_control.xlsx
+++ b/data/final/tables/bootstrap_summary_control.xlsx
@@ -492,19 +492,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2898085.6253058</v>
+        <v>2897995.9243575</v>
       </c>
       <c r="E2" t="n">
-        <v>2897332.681</v>
+        <v>2896029.9795</v>
       </c>
       <c r="F2" t="n">
-        <v>2720240.4348</v>
+        <v>2722354.34795</v>
       </c>
       <c r="G2" t="n">
-        <v>3081412.644475</v>
+        <v>3081745.6311</v>
       </c>
       <c r="H2" t="n">
-        <v>91796.94693387992</v>
+        <v>91978.93302895459</v>
       </c>
       <c r="I2" t="n">
         <v>10000</v>
@@ -527,19 +527,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2895000.698604569</v>
+        <v>2896217.175389451</v>
       </c>
       <c r="E3" t="n">
-        <v>2885416.251114222</v>
+        <v>2886100.079688493</v>
       </c>
       <c r="F3" t="n">
-        <v>2569131.725341174</v>
+        <v>2577404.300096146</v>
       </c>
       <c r="G3" t="n">
-        <v>3266902.545003101</v>
+        <v>3266588.846330027</v>
       </c>
       <c r="H3" t="n">
-        <v>175686.1770983407</v>
+        <v>175211.6722227113</v>
       </c>
       <c r="I3" t="n">
         <v>10000</v>
@@ -562,19 +562,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>8411891591181.093</v>
+        <v>8418769987190.922</v>
       </c>
       <c r="E4" t="n">
-        <v>8325626942234.666</v>
+        <v>8329573670533.555</v>
       </c>
       <c r="F4" t="n">
-        <v>6600437822296.741</v>
+        <v>6643012929132.643</v>
       </c>
       <c r="G4" t="n">
-        <v>10672652238752.44</v>
+        <v>10670602691187.52</v>
       </c>
       <c r="H4" t="n">
-        <v>1025895051886.287</v>
+        <v>1025239164823.266</v>
       </c>
       <c r="I4" t="n">
         <v>10000</v>
@@ -597,19 +597,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>38.2080608</v>
+        <v>38.2019619</v>
       </c>
       <c r="E5" t="n">
-        <v>38.20950000000001</v>
+        <v>38.2</v>
       </c>
       <c r="F5" t="n">
-        <v>37.585</v>
+        <v>37.584</v>
       </c>
       <c r="G5" t="n">
-        <v>38.834</v>
+        <v>38.829</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3169435773548387</v>
+        <v>0.319358947678214</v>
       </c>
       <c r="I5" t="n">
         <v>10000</v>
@@ -632,19 +632,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.01955647892116</v>
+        <v>10.01989120295368</v>
       </c>
       <c r="E6" t="n">
-        <v>10.02088699547729</v>
+        <v>10.01611429375124</v>
       </c>
       <c r="F6" t="n">
-        <v>9.510098721701999</v>
+        <v>9.527585685237206</v>
       </c>
       <c r="G6" t="n">
-        <v>10.53111430445221</v>
+        <v>10.54105370979639</v>
       </c>
       <c r="H6" t="n">
-        <v>0.261825507435799</v>
+        <v>0.2586453820925623</v>
       </c>
       <c r="I6" t="n">
         <v>10000</v>
@@ -667,19 +667,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>100.4600577753754</v>
+        <v>100.465110462963</v>
       </c>
       <c r="E7" t="n">
-        <v>100.4181761761762</v>
+        <v>100.3225455455455</v>
       </c>
       <c r="F7" t="n">
-        <v>90.44197770270269</v>
+        <v>90.77488901401402</v>
       </c>
       <c r="G7" t="n">
-        <v>110.9043684934935</v>
+        <v>111.1138133133133</v>
       </c>
       <c r="H7" t="n">
-        <v>5.249605331010418</v>
+        <v>5.190051708918254</v>
       </c>
       <c r="I7" t="n">
         <v>10000</v>
@@ -702,19 +702,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.492966296666667</v>
+        <v>2.491360781666667</v>
       </c>
       <c r="E8" t="n">
-        <v>2.488183333333333</v>
+        <v>2.487391666666666</v>
       </c>
       <c r="F8" t="n">
-        <v>2.322933333333333</v>
+        <v>2.322883333333333</v>
       </c>
       <c r="G8" t="n">
-        <v>2.690385</v>
+        <v>2.68352375</v>
       </c>
       <c r="H8" t="n">
-        <v>0.09341498496835558</v>
+        <v>0.09184026051559874</v>
       </c>
       <c r="I8" t="n">
         <v>10000</v>
@@ -737,19 +737,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.879746124523172</v>
+        <v>2.873133730368466</v>
       </c>
       <c r="E9" t="n">
-        <v>2.873555218745019</v>
+        <v>2.867405620059029</v>
       </c>
       <c r="F9" t="n">
-        <v>1.975028119964702</v>
+        <v>1.968103108579209</v>
       </c>
       <c r="G9" t="n">
-        <v>3.847314070868554</v>
+        <v>3.803538923503532</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4820223492670366</v>
+        <v>0.4736892857578966</v>
       </c>
       <c r="I9" t="n">
         <v>10000</v>
@@ -772,19 +772,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8.52526005234462</v>
+        <v>8.479256533868895</v>
       </c>
       <c r="E10" t="n">
-        <v>8.257319601545989</v>
+        <v>8.22201499207541</v>
       </c>
       <c r="F10" t="n">
-        <v>3.900736074657991</v>
+        <v>3.873429846207319</v>
       </c>
       <c r="G10" t="n">
-        <v>14.80182556012262</v>
+        <v>14.4669083426204</v>
       </c>
       <c r="H10" t="n">
-        <v>2.818626088632025</v>
+        <v>2.761791580796615</v>
       </c>
       <c r="I10" t="n">
         <v>10000</v>
@@ -807,19 +807,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.5880529999999999</v>
+        <v>0.5878383</v>
       </c>
       <c r="E11" t="n">
         <v>0.588</v>
       </c>
       <c r="F11" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.556</v>
       </c>
       <c r="G11" t="n">
-        <v>0.619</v>
+        <v>0.618</v>
       </c>
       <c r="H11" t="n">
-        <v>0.01555842528856137</v>
+        <v>0.01559235919534076</v>
       </c>
       <c r="I11" t="n">
         <v>10000</v>
@@ -842,19 +842,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.4099403</v>
+        <v>0.4101543</v>
       </c>
       <c r="E12" t="n">
         <v>0.41</v>
       </c>
       <c r="F12" t="n">
-        <v>0.379</v>
+        <v>0.38</v>
       </c>
       <c r="G12" t="n">
-        <v>0.4410249999999996</v>
+        <v>0.441</v>
       </c>
       <c r="H12" t="n">
-        <v>0.01553847741376334</v>
+        <v>0.01558544776797294</v>
       </c>
       <c r="I12" t="n">
         <v>10000</v>
@@ -873,11 +873,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>proportion_otros</t>
+          <t>proportion_others</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.002315334025614432</v>
+        <v>0.002311341393206711</v>
       </c>
       <c r="E13" t="n">
         <v>0.002000000000000002</v>
@@ -889,7 +889,7 @@
         <v>0.005000000000000115</v>
       </c>
       <c r="H13" t="n">
-        <v>0.00125821519706031</v>
+        <v>0.001260795523286588</v>
       </c>
       <c r="I13" t="n">
         <v>10000</v>
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.4942098</v>
+        <v>0.493724</v>
       </c>
       <c r="E14" t="n">
         <v>0.494</v>
       </c>
       <c r="F14" t="n">
-        <v>0.464</v>
+        <v>0.463</v>
       </c>
       <c r="G14" t="n">
         <v>0.525</v>
       </c>
       <c r="H14" t="n">
-        <v>0.01568437387715532</v>
+        <v>0.01580503096803009</v>
       </c>
       <c r="I14" t="n">
         <v>10000</v>
@@ -943,11 +943,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>proportion_otros</t>
+          <t>proportion_others</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.5057902000000001</v>
+        <v>0.5062760000000001</v>
       </c>
       <c r="E15" t="n">
         <v>0.506</v>
@@ -956,10 +956,10 @@
         <v>0.475</v>
       </c>
       <c r="G15" t="n">
-        <v>0.536</v>
+        <v>0.5369999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>0.01568437387715532</v>
+        <v>0.01580503096803009</v>
       </c>
       <c r="I15" t="n">
         <v>10000</v>
@@ -982,19 +982,19 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.6668282999999999</v>
+        <v>0.6670725000000001</v>
       </c>
       <c r="E16" t="n">
         <v>0.667</v>
       </c>
       <c r="F16" t="n">
-        <v>0.638</v>
+        <v>0.637</v>
       </c>
       <c r="G16" t="n">
         <v>0.696</v>
       </c>
       <c r="H16" t="n">
-        <v>0.01488551567691548</v>
+        <v>0.01488151167351519</v>
       </c>
       <c r="I16" t="n">
         <v>10000</v>
@@ -1013,11 +1013,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>proportion_otros</t>
+          <t>proportion_others</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.3331717</v>
+        <v>0.3329275</v>
       </c>
       <c r="E17" t="n">
         <v>0.333</v>
@@ -1026,10 +1026,10 @@
         <v>0.304</v>
       </c>
       <c r="G17" t="n">
-        <v>0.362</v>
+        <v>0.363</v>
       </c>
       <c r="H17" t="n">
-        <v>0.01488551567691548</v>
+        <v>0.01488151167351519</v>
       </c>
       <c r="I17" t="n">
         <v>10000</v>
@@ -1052,19 +1052,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.1520853</v>
+        <v>0.1521932</v>
       </c>
       <c r="E18" t="n">
         <v>0.152</v>
       </c>
       <c r="F18" t="n">
-        <v>0.13</v>
+        <v>0.131</v>
       </c>
       <c r="G18" t="n">
         <v>0.175</v>
       </c>
       <c r="H18" t="n">
-        <v>0.01128910839290822</v>
+        <v>0.01132220353947495</v>
       </c>
       <c r="I18" t="n">
         <v>10000</v>
@@ -1087,19 +1087,19 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.3587590433205887</v>
+        <v>0.3588617563731342</v>
       </c>
       <c r="E19" t="n">
         <v>0.35902089075707</v>
       </c>
       <c r="F19" t="n">
-        <v>0.3363034344160047</v>
+        <v>0.3374003556607491</v>
       </c>
       <c r="G19" t="n">
         <v>0.3799671038392666</v>
       </c>
       <c r="H19" t="n">
-        <v>0.01094948057253978</v>
+        <v>0.01097735227710138</v>
       </c>
       <c r="I19" t="n">
         <v>10000</v>
@@ -1122,19 +1122,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.1288279303</v>
+        <v>0.1289022504</v>
       </c>
       <c r="E20" t="n">
         <v>0.128896</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1131</v>
+        <v>0.113839</v>
       </c>
       <c r="G20" t="n">
         <v>0.144375</v>
       </c>
       <c r="H20" t="n">
-        <v>0.007845975925368625</v>
+        <v>0.007868003513727548</v>
       </c>
       <c r="I20" t="n">
         <v>10000</v>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.5543777</v>
+        <v>0.5540385</v>
       </c>
       <c r="E21" t="n">
         <v>0.554</v>
@@ -1169,7 +1169,7 @@
         <v>0.585</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0159356279177732</v>
+        <v>0.01575108337266807</v>
       </c>
       <c r="I21" t="n">
         <v>10000</v>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.4967755727364511</v>
+        <v>0.4968185736684387</v>
       </c>
       <c r="E22" t="n">
         <v>0.4970754469896899</v>
@@ -1204,7 +1204,7 @@
         <v>0.4994707198625361</v>
       </c>
       <c r="H22" t="n">
-        <v>0.001782568407120686</v>
+        <v>0.001753244262705942</v>
       </c>
       <c r="I22" t="n">
         <v>10000</v>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.2467891469</v>
+        <v>0.2468317687</v>
       </c>
       <c r="E23" t="n">
         <v>0.247084</v>
@@ -1239,7 +1239,7 @@
         <v>0.249471</v>
       </c>
       <c r="H23" t="n">
-        <v>0.001768391147468631</v>
+        <v>0.001739431600043366</v>
       </c>
       <c r="I23" t="n">
         <v>10000</v>

</xml_diff>